<commit_message>
feat: support expanded quiz answer options
Allow imported quiz questions to preserve answer choices beyond A-D and cover the flow with an E2E regression test.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/quiz-template.xlsx
+++ b/frontend/public/quiz-template.xlsx
@@ -397,16 +397,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:J11"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
     <col min="3" max="3" width="20.83203125" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
     <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="35.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="70.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="35.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="70.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -426,12 +428,18 @@
         <v>D</v>
       </c>
       <c r="F1" t="str">
+        <v>E</v>
+      </c>
+      <c r="G1" t="str">
+        <v>F</v>
+      </c>
+      <c r="H1" t="str">
         <v>Đáp án đúng</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Loại câu</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>Giải thích</v>
       </c>
     </row>
@@ -452,12 +460,18 @@
         <v>Parafin</v>
       </c>
       <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
         <v>B</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v>Single choice</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>Crospovidon là tá dược siêu rã thường dùng trong viên nén.</v>
       </c>
     </row>
@@ -478,226 +492,285 @@
         <v>Ảnh đại diện</v>
       </c>
       <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
         <v>A;B;C</v>
       </c>
-      <c r="G3" t="str">
+      <c r="I3" t="str">
         <v>Multiple choice</v>
       </c>
-      <c r="H3" t="str">
+      <c r="J3" t="str">
         <v>File cần câu hỏi, các lựa chọn và đáp án đúng; ảnh đại diện không bắt buộc.</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Quiz có thể được xuất ra định dạng nào?</v>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Câu hỏi có xuống dòng:
+Dòng 1: Nội dung dòng 1
+Dòng 2: Nội dung dòng 2
+Dòng 3: Nội dung dòng 3</v>
       </c>
       <c r="B4" t="str">
-        <v>PDF</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Link online</v>
+        <v>Đáp án A</v>
+      </c>
+      <c r="C4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Đáp án B
+có xuống dòng</v>
       </c>
       <c r="D4" t="str">
-        <v>JSON</v>
+        <v>Đáp án C</v>
       </c>
       <c r="E4" t="str">
-        <v>Tất cả đều đúng</v>
+        <v>Đáp án D</v>
       </c>
       <c r="F4" t="str">
-        <v>D</v>
+        <v/>
       </c>
       <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>B</v>
+      </c>
+      <c r="I4" t="str">
         <v>Single choice</v>
       </c>
-      <c r="H4" t="str">
-        <v>Hệ thống hiện ưu tiên link online và JSON, các định dạng khác có thể mở rộng.</v>
+      <c r="J4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Ví dụ câu hỏi và đáp án có xuống dòng.
+Xuống dòng sẽ được giữ nguyên.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2 + 2 = ?</v>
+        <v>Câu hỏi có 6 đáp án - Chọn 1 đáp án đúng?</v>
       </c>
       <c r="B5" t="str">
-        <v>3</v>
+        <v>Đáp án A</v>
       </c>
       <c r="C5" t="str">
-        <v>4</v>
+        <v>Đáp án B</v>
       </c>
       <c r="D5" t="str">
-        <v>5</v>
+        <v>Đáp án C</v>
       </c>
       <c r="E5" t="str">
-        <v>6</v>
+        <v>Đáp án D</v>
       </c>
       <c r="F5" t="str">
-        <v>B</v>
+        <v>Đáp án E</v>
       </c>
       <c r="G5" t="str">
+        <v>Đáp án F (đúng)</v>
+      </c>
+      <c r="H5" t="str">
+        <v>F</v>
+      </c>
+      <c r="I5" t="str">
         <v>Single choice</v>
       </c>
-      <c r="H5" t="str">
-        <v>2 + 2 bằng 4.</v>
+      <c r="J5" t="str">
+        <v>Ví dụ câu hỏi có 6 đáp án (A-F).</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Thủ đô của Việt Nam là?</v>
+        <v>Câu hỏi có 5 đáp án - Chọn nhiều đáp án đúng?</v>
       </c>
       <c r="B6" t="str">
-        <v>Hà Nội</v>
+        <v>Đáp án A (đúng)</v>
       </c>
       <c r="C6" t="str">
-        <v>TP.HCM</v>
+        <v>Đáp án B</v>
       </c>
       <c r="D6" t="str">
-        <v>Đà Nẵng</v>
+        <v>Đáp án C (đúng)</v>
       </c>
       <c r="E6" t="str">
-        <v>Huế</v>
+        <v>Đáp án D</v>
       </c>
       <c r="F6" t="str">
-        <v>A</v>
+        <v>Đáp án E (đúng)</v>
       </c>
       <c r="G6" t="str">
-        <v>Single choice</v>
+        <v/>
       </c>
       <c r="H6" t="str">
-        <v>Hà Nội là thủ đô của Việt Nam.</v>
+        <v>A;C;E</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Multiple choice</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Ví dụ câu hỏi có 5 đáp án và 3 đáp án đúng.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Màu của bầu trời vào ngày nắng thường là?</v>
+        <v>2 + 2 = ?</v>
       </c>
       <c r="B7" t="str">
-        <v>Xanh</v>
+        <v>3</v>
       </c>
       <c r="C7" t="str">
-        <v>Đỏ</v>
+        <v>4</v>
       </c>
       <c r="D7" t="str">
-        <v>Vàng</v>
+        <v>5</v>
       </c>
       <c r="E7" t="str">
-        <v>Tím</v>
+        <v>6</v>
       </c>
       <c r="F7" t="str">
-        <v>A</v>
+        <v/>
       </c>
       <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>B</v>
+      </c>
+      <c r="I7" t="str">
         <v>Single choice</v>
       </c>
-      <c r="H7" t="str">
-        <v>Ánh sáng tán xạ khiến bầu trời thường có màu xanh.</v>
+      <c r="J7" t="str">
+        <v>2 + 2 bằng 4.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Python là gì?</v>
+        <v>Thủ đô của Việt Nam là?</v>
       </c>
       <c r="B8" t="str">
-        <v>Ngôn ngữ lập trình</v>
+        <v>Hà Nội</v>
       </c>
       <c r="C8" t="str">
-        <v>Con rắn</v>
+        <v>TP.HCM</v>
       </c>
       <c r="D8" t="str">
-        <v>Thương hiệu</v>
+        <v>Đà Nẵng</v>
       </c>
       <c r="E8" t="str">
-        <v>Tất cả đều đúng</v>
+        <v>Huế</v>
       </c>
       <c r="F8" t="str">
-        <v>D</v>
+        <v/>
       </c>
       <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>A</v>
+      </c>
+      <c r="I8" t="str">
         <v>Single choice</v>
       </c>
-      <c r="H8" t="str">
-        <v>Python vừa là tên ngôn ngữ lập trình, vừa là tên một loài rắn và có thể là tên thương hiệu.</v>
+      <c r="J8" t="str">
+        <v>Hà Nội là thủ đô của Việt Nam.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>React là?</v>
+        <v>Màu của bầu trời vào ngày nắng thường là?</v>
       </c>
       <c r="B9" t="str">
-        <v>Library JavaScript</v>
+        <v>Xanh</v>
       </c>
       <c r="C9" t="str">
-        <v>Framework</v>
+        <v>Đỏ</v>
       </c>
       <c r="D9" t="str">
-        <v>Database</v>
+        <v>Vàng</v>
       </c>
       <c r="E9" t="str">
-        <v>Server</v>
+        <v>Tím</v>
       </c>
       <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
         <v>A</v>
       </c>
-      <c r="G9" t="str">
+      <c r="I9" t="str">
         <v>Single choice</v>
       </c>
-      <c r="H9" t="str">
-        <v>React là thư viện JavaScript để xây dựng giao diện người dùng.</v>
+      <c r="J9" t="str">
+        <v>Ánh sáng tán xạ khiến bầu trời thường có màu xanh.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MongoDB là?</v>
+        <v>Python là gì?</v>
       </c>
       <c r="B10" t="str">
-        <v>SQL Database</v>
+        <v>Ngôn ngữ lập trình</v>
       </c>
       <c r="C10" t="str">
-        <v>NoSQL Database</v>
+        <v>Con rắn</v>
       </c>
       <c r="D10" t="str">
-        <v>Programming Language</v>
+        <v>Thương hiệu</v>
       </c>
       <c r="E10" t="str">
-        <v>Framework</v>
+        <v>Tất cả đều đúng</v>
       </c>
       <c r="F10" t="str">
-        <v>B</v>
+        <v/>
       </c>
       <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v>D</v>
+      </c>
+      <c r="I10" t="str">
         <v>Single choice</v>
       </c>
-      <c r="H10" t="str">
-        <v>MongoDB là cơ sở dữ liệu NoSQL hướng document.</v>
+      <c r="J10" t="str">
+        <v>Python vừa là tên ngôn ngữ lập trình, vừa là tên một loài rắn và có thể là tên thương hiệu.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>1 + 1 = ?</v>
+        <v>React là?</v>
       </c>
       <c r="B11" t="str">
-        <v>1</v>
+        <v>Library JavaScript</v>
       </c>
       <c r="C11" t="str">
-        <v>2</v>
+        <v>Framework</v>
       </c>
       <c r="D11" t="str">
-        <v>3</v>
+        <v>Database</v>
       </c>
       <c r="E11" t="str">
-        <v>4</v>
+        <v>Server</v>
       </c>
       <c r="F11" t="str">
-        <v>B</v>
+        <v/>
       </c>
       <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v>A</v>
+      </c>
+      <c r="I11" t="str">
         <v>Single choice</v>
       </c>
-      <c r="H11" t="str">
-        <v>1 + 1 bằng 2.</v>
+      <c r="J11" t="str">
+        <v>React là thư viện JavaScript để xây dựng giao diện người dùng.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>